<commit_message>
Updated EGY_grids_kan10 model - 2026-06-18 23:43
</commit_message>
<xml_diff>
--- a/VerveStacks_EGY_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_EGY_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_EGY_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A748A323-3624-44A7-9B99-85F5278BDB4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CFC8BED-F6E4-4D58-8924-72AFF88FDC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="70" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5424" uniqueCount="722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5423" uniqueCount="722">
   <si>
     <t>Unit</t>
   </si>
@@ -19753,7 +19753,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C19CC6EB-F898-4E1F-ACDF-67B835EB4CDD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC7E7885-8739-40CE-8B24-10E5CA518FA7}">
   <dimension ref="B9:H116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21911,7 +21911,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04445D07-B949-4070-94FA-FB0A1603F4F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{220A3E16-C470-4508-97C1-48D2A9168DFB}">
   <dimension ref="B9:L116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -25141,9 +25141,6 @@
       <c r="N3" t="s">
         <v>63</v>
       </c>
-      <c r="Q3" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" t="s">

</xml_diff>